<commit_message>
10 board costs removed from client BOM #3
</commit_message>
<xml_diff>
--- a/Design-Files/DBS-Stepper-Module/BOM/Client-BOM-v1.0.xlsx
+++ b/Design-Files/DBS-Stepper-Module/BOM/Client-BOM-v1.0.xlsx
@@ -1462,7 +1462,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1562,24 +1562,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1630,9 +1617,6 @@
     </xf>
     <xf numFmtId="166" fontId="12" fillId="3" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1702,11 +1686,11 @@
     <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="15" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1995,7 +1979,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O170"/>
+  <dimension ref="A1:O169"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="10" customWidth="1"/>
@@ -2039,90 +2023,90 @@
         <v>0</v>
       </c>
       <c r="E2" s="4"/>
-      <c r="F2" s="39" t="s">
+      <c r="F2" s="38" t="s">
         <v>391</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
     </row>
     <row r="3" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="8"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="38" t="s">
+      <c r="C3" s="25"/>
+      <c r="D3" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="27"/>
-      <c r="F3" s="40" t="s">
+      <c r="E3" s="26"/>
+      <c r="F3" s="39" t="s">
         <v>392</v>
       </c>
-      <c r="G3" s="29"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="24"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
     </row>
     <row r="4" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="8"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="24"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="24"/>
-      <c r="M4" s="24"/>
-      <c r="N4" s="24"/>
-      <c r="O4" s="24"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
     </row>
     <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="9"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="35"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="35"/>
-      <c r="K5" s="35"/>
-      <c r="L5" s="35"/>
-      <c r="M5" s="35"/>
-      <c r="N5" s="35"/>
-      <c r="O5" s="35"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="34"/>
+      <c r="K5" s="34"/>
+      <c r="L5" s="34"/>
+      <c r="M5" s="34"/>
+      <c r="N5" s="34"/>
+      <c r="O5" s="34"/>
     </row>
     <row r="6" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="35"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="35"/>
-      <c r="K6" s="35"/>
-      <c r="L6" s="35"/>
-      <c r="M6" s="35"/>
-      <c r="N6" s="35"/>
-      <c r="O6" s="35"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="34"/>
+      <c r="L6" s="34"/>
+      <c r="M6" s="34"/>
+      <c r="N6" s="34"/>
+      <c r="O6" s="34"/>
     </row>
     <row r="7" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
@@ -2175,7 +2159,7 @@
         <f>ROW(B8) - ROW($B$7)</f>
         <v>1</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="21" t="s">
         <v>4</v>
       </c>
       <c r="D8" s="14" t="s">
@@ -2208,7 +2192,7 @@
       <c r="M8" s="15">
         <v>7.4250000000000002E-3</v>
       </c>
-      <c r="N8" s="48">
+      <c r="N8" s="46">
         <f>M8*L8</f>
         <v>0.14849999999999999</v>
       </c>
@@ -2220,44 +2204,44 @@
         <f t="shared" ref="B9:B77" si="0">ROW(B9) - ROW($B$7)</f>
         <v>2</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="20" t="s">
+      <c r="E9" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="F9" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="H9" s="20" t="s">
+      <c r="H9" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="I9" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J9" s="20" t="s">
+      <c r="I9" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J9" s="19" t="s">
         <v>296</v>
       </c>
-      <c r="K9" s="20" t="s">
+      <c r="K9" s="19" t="s">
         <v>351</v>
       </c>
-      <c r="L9" s="20">
+      <c r="L9" s="19">
         <v>2</v>
       </c>
-      <c r="M9" s="21">
+      <c r="M9" s="20">
         <v>0.222525</v>
       </c>
-      <c r="N9" s="48">
+      <c r="N9" s="46">
         <f t="shared" ref="N9:N72" si="1">M9*L9</f>
         <v>0.44505</v>
       </c>
-      <c r="O9" s="20"/>
+      <c r="O9" s="19"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
@@ -2265,7 +2249,7 @@
         <f>ROW(B10) - ROW($B$7)</f>
         <v>3</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="21" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="14" t="s">
@@ -2277,7 +2261,7 @@
       <c r="F10" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="G10" s="41" t="s">
+      <c r="G10" s="40" t="s">
         <v>213</v>
       </c>
       <c r="H10" s="14" t="s">
@@ -2298,7 +2282,7 @@
       <c r="M10" s="15">
         <v>6.3E-3</v>
       </c>
-      <c r="N10" s="48">
+      <c r="N10" s="46">
         <f t="shared" si="1"/>
         <v>6.3E-3</v>
       </c>
@@ -2310,44 +2294,44 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="F11" s="20" t="s">
+      <c r="F11" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="H11" s="20" t="s">
+      <c r="H11" s="19" t="s">
         <v>266</v>
       </c>
-      <c r="I11" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J11" s="20" t="s">
+      <c r="I11" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J11" s="19" t="s">
         <v>297</v>
       </c>
-      <c r="K11" s="20" t="s">
+      <c r="K11" s="19" t="s">
         <v>353</v>
       </c>
-      <c r="L11" s="20">
+      <c r="L11" s="19">
         <v>3</v>
       </c>
-      <c r="M11" s="21">
+      <c r="M11" s="20">
         <v>0.64529999999999998</v>
       </c>
-      <c r="N11" s="48">
+      <c r="N11" s="46">
         <f t="shared" si="1"/>
         <v>1.9359</v>
       </c>
-      <c r="O11" s="20"/>
+      <c r="O11" s="19"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
@@ -2355,7 +2339,7 @@
         <f>ROW(B12) - ROW($B$7)</f>
         <v>5</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="21" t="s">
         <v>4</v>
       </c>
       <c r="D12" s="14" t="s">
@@ -2388,7 +2372,7 @@
       <c r="M12" s="15">
         <v>4.725E-3</v>
       </c>
-      <c r="N12" s="48">
+      <c r="N12" s="46">
         <f t="shared" si="1"/>
         <v>4.725E-3</v>
       </c>
@@ -2400,44 +2384,44 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="E13" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="F13" s="20" t="s">
+      <c r="F13" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="H13" s="20" t="s">
+      <c r="H13" s="19" t="s">
         <v>267</v>
       </c>
-      <c r="I13" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J13" s="20" t="s">
+      <c r="I13" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J13" s="19" t="s">
         <v>299</v>
       </c>
-      <c r="K13" s="20" t="s">
+      <c r="K13" s="19" t="s">
         <v>355</v>
       </c>
-      <c r="L13" s="20">
+      <c r="L13" s="19">
         <v>3</v>
       </c>
-      <c r="M13" s="21">
+      <c r="M13" s="20">
         <v>1.0124999999999999E-2</v>
       </c>
-      <c r="N13" s="48">
+      <c r="N13" s="46">
         <f t="shared" si="1"/>
         <v>3.0374999999999996E-2</v>
       </c>
-      <c r="O13" s="20"/>
+      <c r="O13" s="19"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
@@ -2445,7 +2429,7 @@
         <f>ROW(B14) - ROW($B$7)</f>
         <v>7</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="21" t="s">
         <v>4</v>
       </c>
       <c r="D14" s="14" t="s">
@@ -2457,7 +2441,7 @@
       <c r="F14" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="G14" s="41" t="s">
+      <c r="G14" s="40" t="s">
         <v>217</v>
       </c>
       <c r="H14" s="14" t="s">
@@ -2478,7 +2462,7 @@
       <c r="M14" s="15">
         <v>2.0924999999999999E-2</v>
       </c>
-      <c r="N14" s="48">
+      <c r="N14" s="46">
         <f t="shared" si="1"/>
         <v>2.0924999999999999E-2</v>
       </c>
@@ -2490,44 +2474,44 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D15" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="E15" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="F15" s="20" t="s">
+      <c r="F15" s="19" t="s">
         <v>395</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="G15" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="H15" s="20" t="s">
+      <c r="H15" s="19" t="s">
         <v>268</v>
       </c>
-      <c r="I15" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J15" s="20" t="s">
+      <c r="I15" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J15" s="19" t="s">
         <v>300</v>
       </c>
-      <c r="K15" s="20" t="s">
+      <c r="K15" s="19" t="s">
         <v>353</v>
       </c>
-      <c r="L15" s="20">
+      <c r="L15" s="19">
         <v>1</v>
       </c>
-      <c r="M15" s="21">
+      <c r="M15" s="20">
         <v>7.4024999999999994E-2</v>
       </c>
-      <c r="N15" s="48">
+      <c r="N15" s="46">
         <f t="shared" si="1"/>
         <v>7.4024999999999994E-2</v>
       </c>
-      <c r="O15" s="20"/>
+      <c r="O15" s="19"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
@@ -2535,7 +2519,7 @@
         <f>ROW(B16) - ROW($B$7)</f>
         <v>9</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="22" t="s">
         <v>4</v>
       </c>
       <c r="D16" s="14" t="s">
@@ -2547,7 +2531,7 @@
       <c r="F16" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="G16" s="41" t="s">
+      <c r="G16" s="40" t="s">
         <v>218</v>
       </c>
       <c r="H16" s="14" t="s">
@@ -2568,7 +2552,7 @@
       <c r="M16" s="15">
         <v>2.835E-2</v>
       </c>
-      <c r="N16" s="48">
+      <c r="N16" s="46">
         <f t="shared" si="1"/>
         <v>5.67E-2</v>
       </c>
@@ -2580,44 +2564,44 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D17" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="20" t="s">
+      <c r="E17" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="F17" s="20" t="s">
+      <c r="F17" s="19" t="s">
         <v>395</v>
       </c>
-      <c r="G17" s="20" t="s">
+      <c r="G17" s="19" t="s">
         <v>172</v>
       </c>
-      <c r="H17" s="20" t="s">
+      <c r="H17" s="19" t="s">
         <v>268</v>
       </c>
-      <c r="I17" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J17" s="20" t="s">
+      <c r="I17" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J17" s="19" t="s">
         <v>301</v>
       </c>
-      <c r="K17" s="20" t="s">
+      <c r="K17" s="19" t="s">
         <v>358</v>
       </c>
-      <c r="L17" s="20">
+      <c r="L17" s="19">
         <v>2</v>
       </c>
-      <c r="M17" s="21">
+      <c r="M17" s="20">
         <v>0.12847500000000001</v>
       </c>
-      <c r="N17" s="48">
+      <c r="N17" s="46">
         <f t="shared" si="1"/>
         <v>0.25695000000000001</v>
       </c>
-      <c r="O17" s="20"/>
+      <c r="O17" s="19"/>
     </row>
     <row r="18" spans="1:15" ht="24" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
@@ -2625,7 +2609,7 @@
         <f>ROW(B18) - ROW($B$7)</f>
         <v>11</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="21" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="14" t="s">
@@ -2643,7 +2627,7 @@
       <c r="H18" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I18" s="20" t="s">
+      <c r="I18" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J18" s="14" t="s">
@@ -2658,7 +2642,7 @@
       <c r="M18" s="15">
         <v>2.07E-2</v>
       </c>
-      <c r="N18" s="48">
+      <c r="N18" s="46">
         <f t="shared" si="1"/>
         <v>4.1399999999999999E-2</v>
       </c>
@@ -2670,44 +2654,44 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="20" t="s">
+      <c r="E19" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="F19" s="20" t="s">
+      <c r="F19" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="G19" s="20" t="s">
+      <c r="G19" s="19" t="s">
         <v>220</v>
       </c>
-      <c r="H19" s="20" t="s">
+      <c r="H19" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="I19" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J19" s="20" t="s">
+      <c r="I19" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J19" s="19" t="s">
         <v>303</v>
       </c>
-      <c r="K19" s="20" t="s">
+      <c r="K19" s="19" t="s">
         <v>360</v>
       </c>
-      <c r="L19" s="20">
+      <c r="L19" s="19">
         <v>1</v>
       </c>
-      <c r="M19" s="21">
+      <c r="M19" s="20">
         <v>6.3E-3</v>
       </c>
-      <c r="N19" s="48">
+      <c r="N19" s="46">
         <f t="shared" si="1"/>
         <v>6.3E-3</v>
       </c>
-      <c r="O19" s="20"/>
+      <c r="O19" s="19"/>
     </row>
     <row r="20" spans="1:15" ht="24" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
@@ -2715,7 +2699,7 @@
         <f>ROW(B20) - ROW($B$7)</f>
         <v>13</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="21" t="s">
         <v>4</v>
       </c>
       <c r="D20" s="14" t="s">
@@ -2733,7 +2717,7 @@
       <c r="H20" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I20" s="20" t="s">
+      <c r="I20" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J20" s="14" t="s">
@@ -2748,7 +2732,7 @@
       <c r="M20" s="15">
         <v>1.755E-2</v>
       </c>
-      <c r="N20" s="48">
+      <c r="N20" s="46">
         <f t="shared" si="1"/>
         <v>7.0199999999999999E-2</v>
       </c>
@@ -2760,44 +2744,44 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F21" s="20" t="s">
+      <c r="F21" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="G21" s="20" t="s">
+      <c r="G21" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="H21" s="20" t="s">
+      <c r="H21" s="19" t="s">
         <v>267</v>
       </c>
-      <c r="I21" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J21" s="20" t="s">
+      <c r="I21" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J21" s="19" t="s">
         <v>305</v>
       </c>
-      <c r="K21" s="20" t="s">
+      <c r="K21" s="19" t="s">
         <v>362</v>
       </c>
-      <c r="L21" s="20">
+      <c r="L21" s="19">
         <v>4</v>
       </c>
-      <c r="M21" s="21">
+      <c r="M21" s="20">
         <v>8.5500000000000003E-3</v>
       </c>
-      <c r="N21" s="48">
+      <c r="N21" s="46">
         <f t="shared" si="1"/>
         <v>3.4200000000000001E-2</v>
       </c>
-      <c r="O21" s="20"/>
+      <c r="O21" s="19"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
@@ -2805,7 +2789,7 @@
         <f>ROW(B22) - ROW($B$7)</f>
         <v>15</v>
       </c>
-      <c r="C22" s="22" t="s">
+      <c r="C22" s="21" t="s">
         <v>4</v>
       </c>
       <c r="D22" s="14" t="s">
@@ -2823,7 +2807,7 @@
       <c r="H22" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I22" s="20" t="s">
+      <c r="I22" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J22" s="14" t="s">
@@ -2838,7 +2822,7 @@
       <c r="M22" s="15">
         <v>4.7024999999999997E-2</v>
       </c>
-      <c r="N22" s="48">
+      <c r="N22" s="46">
         <f t="shared" si="1"/>
         <v>9.4049999999999995E-2</v>
       </c>
@@ -2850,44 +2834,44 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="20" t="s">
+      <c r="D23" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="E23" s="20" t="s">
+      <c r="E23" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="F23" s="20" t="s">
+      <c r="F23" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="G23" s="20" t="s">
+      <c r="G23" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="H23" s="20" t="s">
+      <c r="H23" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="I23" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J23" s="20" t="s">
+      <c r="I23" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J23" s="19" t="s">
         <v>307</v>
       </c>
-      <c r="K23" s="20" t="s">
+      <c r="K23" s="19" t="s">
         <v>364</v>
       </c>
-      <c r="L23" s="20">
+      <c r="L23" s="19">
         <v>1</v>
       </c>
-      <c r="M23" s="21">
+      <c r="M23" s="20">
         <v>2.1150000000000002E-2</v>
       </c>
-      <c r="N23" s="48">
+      <c r="N23" s="46">
         <f t="shared" si="1"/>
         <v>2.1150000000000002E-2</v>
       </c>
-      <c r="O23" s="20"/>
+      <c r="O23" s="19"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
@@ -2895,7 +2879,7 @@
         <f>ROW(B24) - ROW($B$7)</f>
         <v>17</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="C24" s="22" t="s">
         <v>4</v>
       </c>
       <c r="D24" s="14" t="s">
@@ -2928,7 +2912,7 @@
       <c r="M24" s="15">
         <v>9.9225000000000008E-2</v>
       </c>
-      <c r="N24" s="48">
+      <c r="N24" s="46">
         <f t="shared" si="1"/>
         <v>9.9225000000000008E-2</v>
       </c>
@@ -2940,44 +2924,44 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="E25" s="20" t="s">
+      <c r="E25" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="F25" s="20" t="s">
+      <c r="F25" s="19" t="s">
         <v>175</v>
       </c>
-      <c r="G25" s="20" t="s">
+      <c r="G25" s="19" t="s">
         <v>226</v>
       </c>
-      <c r="H25" s="20" t="s">
+      <c r="H25" s="19" t="s">
         <v>269</v>
       </c>
-      <c r="I25" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J25" s="20" t="s">
+      <c r="I25" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J25" s="19" t="s">
         <v>308</v>
       </c>
       <c r="K25" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L25" s="20">
+      <c r="L25" s="19">
         <v>1</v>
       </c>
-      <c r="M25" s="21">
+      <c r="M25" s="20">
         <v>7.8299999999999995E-2</v>
       </c>
-      <c r="N25" s="48">
+      <c r="N25" s="46">
         <f t="shared" si="1"/>
         <v>7.8299999999999995E-2</v>
       </c>
-      <c r="O25" s="20"/>
+      <c r="O25" s="19"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
@@ -2985,7 +2969,7 @@
         <f>ROW(B26) - ROW($B$7)</f>
         <v>19</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="21" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="14" t="s">
@@ -3018,7 +3002,7 @@
       <c r="M26" s="15">
         <v>0.2475</v>
       </c>
-      <c r="N26" s="48">
+      <c r="N26" s="46">
         <f t="shared" si="1"/>
         <v>0.2475</v>
       </c>
@@ -3030,25 +3014,25 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C27" s="22" t="s">
+      <c r="C27" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D27" s="20" t="s">
+      <c r="D27" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E27" s="20" t="s">
+      <c r="E27" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="F27" s="20" t="s">
+      <c r="F27" s="19" t="s">
         <v>175</v>
       </c>
-      <c r="G27" s="20" t="s">
+      <c r="G27" s="19" t="s">
         <v>228</v>
       </c>
-      <c r="H27" s="20" t="s">
+      <c r="H27" s="19" t="s">
         <v>271</v>
       </c>
-      <c r="I27" s="20" t="s">
+      <c r="I27" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J27" s="14" t="s">
@@ -3057,17 +3041,17 @@
       <c r="K27" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L27" s="20">
+      <c r="L27" s="19">
         <v>1</v>
       </c>
-      <c r="M27" s="21">
+      <c r="M27" s="20">
         <v>7.7399999999999997E-2</v>
       </c>
-      <c r="N27" s="48">
+      <c r="N27" s="46">
         <f t="shared" si="1"/>
         <v>7.7399999999999997E-2</v>
       </c>
-      <c r="O27" s="20"/>
+      <c r="O27" s="19"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
@@ -3075,7 +3059,7 @@
         <f>ROW(B28) - ROW($B$7)</f>
         <v>21</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="21" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="14" t="s">
@@ -3108,7 +3092,7 @@
       <c r="M28" s="15">
         <v>3.2625000000000001E-2</v>
       </c>
-      <c r="N28" s="48">
+      <c r="N28" s="46">
         <f t="shared" si="1"/>
         <v>6.5250000000000002E-2</v>
       </c>
@@ -3120,44 +3104,44 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C29" s="23" t="s">
+      <c r="C29" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="D29" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="E29" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="F29" s="20" t="s">
+      <c r="F29" s="19" t="s">
         <v>395</v>
       </c>
-      <c r="G29" s="20" t="s">
+      <c r="G29" s="19" t="s">
         <v>398</v>
       </c>
-      <c r="H29" s="20" t="s">
+      <c r="H29" s="19" t="s">
         <v>272</v>
       </c>
-      <c r="I29" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J29" s="20" t="s">
+      <c r="I29" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J29" s="19" t="s">
         <v>230</v>
       </c>
       <c r="K29" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L29" s="20">
+      <c r="L29" s="19">
         <v>1</v>
       </c>
-      <c r="M29" s="21">
+      <c r="M29" s="20">
         <v>0.145125</v>
       </c>
-      <c r="N29" s="48">
+      <c r="N29" s="46">
         <f t="shared" si="1"/>
         <v>0.145125</v>
       </c>
-      <c r="O29" s="20"/>
+      <c r="O29" s="19"/>
     </row>
     <row r="30" spans="1:15" ht="48" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
@@ -3165,7 +3149,7 @@
         <f>ROW(B30) - ROW($B$7)</f>
         <v>23</v>
       </c>
-      <c r="C30" s="22" t="s">
+      <c r="C30" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D30" s="14" t="s">
@@ -3183,7 +3167,7 @@
       <c r="H30" s="14" t="s">
         <v>273</v>
       </c>
-      <c r="I30" s="20" t="s">
+      <c r="I30" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J30" s="14" t="s">
@@ -3198,7 +3182,7 @@
       <c r="M30" s="15">
         <v>0.56182500000000002</v>
       </c>
-      <c r="N30" s="48">
+      <c r="N30" s="46">
         <f t="shared" si="1"/>
         <v>0.56182500000000002</v>
       </c>
@@ -3210,44 +3194,44 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="C31" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="E31" s="20" t="s">
+      <c r="E31" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="F31" s="20" t="s">
+      <c r="F31" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="G31" s="20" t="s">
+      <c r="G31" s="19" t="s">
         <v>231</v>
       </c>
-      <c r="H31" s="20" t="s">
+      <c r="H31" s="19" t="s">
         <v>274</v>
       </c>
-      <c r="I31" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J31" s="20" t="s">
+      <c r="I31" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J31" s="19" t="s">
         <v>312</v>
       </c>
       <c r="K31" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L31" s="20">
+      <c r="L31" s="19">
         <v>2</v>
       </c>
-      <c r="M31" s="21">
+      <c r="M31" s="20">
         <v>0.113625</v>
       </c>
-      <c r="N31" s="48">
+      <c r="N31" s="46">
         <f t="shared" si="1"/>
         <v>0.22725000000000001</v>
       </c>
-      <c r="O31" s="20"/>
+      <c r="O31" s="19"/>
     </row>
     <row r="32" spans="1:15" ht="48" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
@@ -3255,7 +3239,7 @@
         <f>ROW(B32) - ROW($B$7)</f>
         <v>25</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="C32" s="21" t="s">
         <v>12</v>
       </c>
       <c r="D32" s="14" t="s">
@@ -3273,7 +3257,7 @@
       <c r="H32" s="14" t="s">
         <v>275</v>
       </c>
-      <c r="I32" s="20" t="s">
+      <c r="I32" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J32" s="14" t="s">
@@ -3288,7 +3272,7 @@
       <c r="M32" s="15">
         <v>8.0325000000000008E-2</v>
       </c>
-      <c r="N32" s="48">
+      <c r="N32" s="46">
         <f t="shared" si="1"/>
         <v>8.0325000000000008E-2</v>
       </c>
@@ -3300,44 +3284,44 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C33" s="23" t="s">
+      <c r="C33" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="D33" s="20" t="s">
+      <c r="D33" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="E33" s="20" t="s">
+      <c r="E33" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="F33" s="20" t="s">
+      <c r="F33" s="19" t="s">
         <v>395</v>
       </c>
-      <c r="G33" s="20" t="s">
+      <c r="G33" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="H33" s="20" t="s">
+      <c r="H33" s="19" t="s">
         <v>276</v>
       </c>
-      <c r="I33" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J33" s="20" t="s">
+      <c r="I33" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J33" s="19" t="s">
         <v>314</v>
       </c>
       <c r="K33" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L33" s="20">
+      <c r="L33" s="19">
         <v>1</v>
       </c>
-      <c r="M33" s="21">
+      <c r="M33" s="20">
         <v>0.33772500000000005</v>
       </c>
-      <c r="N33" s="48">
+      <c r="N33" s="46">
         <f t="shared" si="1"/>
         <v>0.33772500000000005</v>
       </c>
-      <c r="O33" s="20"/>
+      <c r="O33" s="19"/>
     </row>
     <row r="34" spans="1:15" ht="48" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
@@ -3345,7 +3329,7 @@
         <f>ROW(B34) - ROW($B$7)</f>
         <v>27</v>
       </c>
-      <c r="C34" s="22" t="s">
+      <c r="C34" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D34" s="14" t="s">
@@ -3354,7 +3338,7 @@
       <c r="E34" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="F34" s="20" t="s">
+      <c r="F34" s="19" t="s">
         <v>395</v>
       </c>
       <c r="G34" s="14" t="s">
@@ -3363,7 +3347,7 @@
       <c r="H34" s="14" t="s">
         <v>277</v>
       </c>
-      <c r="I34" s="20" t="s">
+      <c r="I34" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J34" s="14" t="s">
@@ -3378,7 +3362,7 @@
       <c r="M34" s="15">
         <v>0.35752500000000004</v>
       </c>
-      <c r="N34" s="48">
+      <c r="N34" s="46">
         <f t="shared" si="1"/>
         <v>0.35752500000000004</v>
       </c>
@@ -3390,44 +3374,44 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C35" s="23" t="s">
+      <c r="C35" s="22" t="s">
         <v>390</v>
       </c>
-      <c r="D35" s="20" t="s">
+      <c r="D35" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="E35" s="20" t="s">
+      <c r="E35" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="F35" s="20" t="s">
+      <c r="F35" s="19" t="s">
         <v>395</v>
       </c>
-      <c r="G35" s="20" t="s">
+      <c r="G35" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="H35" s="20" t="s">
+      <c r="H35" s="19" t="s">
         <v>278</v>
       </c>
-      <c r="I35" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J35" s="20" t="s">
+      <c r="I35" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J35" s="19" t="s">
         <v>316</v>
       </c>
       <c r="K35" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L35" s="20">
+      <c r="L35" s="19">
         <v>1</v>
       </c>
-      <c r="M35" s="21">
+      <c r="M35" s="20">
         <v>0.82845000000000002</v>
       </c>
-      <c r="N35" s="48">
+      <c r="N35" s="46">
         <f t="shared" si="1"/>
         <v>0.82845000000000002</v>
       </c>
-      <c r="O35" s="20"/>
+      <c r="O35" s="19"/>
     </row>
     <row r="36" spans="1:15" ht="48" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
@@ -3435,7 +3419,7 @@
         <f>ROW(B36) - ROW($B$7)</f>
         <v>29</v>
       </c>
-      <c r="C36" s="22" t="s">
+      <c r="C36" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D36" s="14" t="s">
@@ -3444,7 +3428,7 @@
       <c r="E36" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="F36" s="20" t="s">
+      <c r="F36" s="19" t="s">
         <v>395</v>
       </c>
       <c r="G36" s="14" t="s">
@@ -3453,7 +3437,7 @@
       <c r="H36" s="14" t="s">
         <v>277</v>
       </c>
-      <c r="I36" s="20" t="s">
+      <c r="I36" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J36" s="14" t="s">
@@ -3468,7 +3452,7 @@
       <c r="M36" s="15">
         <v>0.35640000000000005</v>
       </c>
-      <c r="N36" s="48">
+      <c r="N36" s="46">
         <f t="shared" si="1"/>
         <v>0.35640000000000005</v>
       </c>
@@ -3480,44 +3464,44 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C37" s="23" t="s">
+      <c r="C37" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="D37" s="20" t="s">
+      <c r="D37" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="E37" s="20" t="s">
+      <c r="E37" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="F37" s="20" t="s">
+      <c r="F37" s="19" t="s">
         <v>185</v>
       </c>
-      <c r="G37" s="20" t="s">
+      <c r="G37" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="H37" s="20" t="s">
+      <c r="H37" s="19" t="s">
         <v>275</v>
       </c>
-      <c r="I37" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J37" s="20" t="s">
+      <c r="I37" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J37" s="19" t="s">
         <v>318</v>
       </c>
       <c r="K37" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L37" s="20">
+      <c r="L37" s="19">
         <v>1</v>
       </c>
-      <c r="M37" s="21">
+      <c r="M37" s="20">
         <v>4.2300000000000004E-2</v>
       </c>
-      <c r="N37" s="48">
+      <c r="N37" s="46">
         <f t="shared" si="1"/>
         <v>4.2300000000000004E-2</v>
       </c>
-      <c r="O37" s="20"/>
+      <c r="O37" s="19"/>
     </row>
     <row r="38" spans="1:15" ht="24" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
@@ -3525,7 +3509,7 @@
         <f>ROW(B38) - ROW($B$7)</f>
         <v>31</v>
       </c>
-      <c r="C38" s="22" t="s">
+      <c r="C38" s="21" t="s">
         <v>13</v>
       </c>
       <c r="D38" s="14" t="s">
@@ -3543,7 +3527,7 @@
       <c r="H38" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="I38" s="20" t="s">
+      <c r="I38" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J38" s="14" t="s">
@@ -3558,7 +3542,7 @@
       <c r="M38" s="15">
         <v>1.5246</v>
       </c>
-      <c r="N38" s="48">
+      <c r="N38" s="46">
         <f t="shared" si="1"/>
         <v>1.5246</v>
       </c>
@@ -3570,44 +3554,44 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C39" s="23" t="s">
+      <c r="C39" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="D39" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="E39" s="20" t="s">
+      <c r="E39" s="19" t="s">
         <v>130</v>
       </c>
       <c r="F39" s="14" t="s">
         <v>395</v>
       </c>
-      <c r="G39" s="20" t="s">
+      <c r="G39" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="H39" s="20" t="s">
+      <c r="H39" s="19" t="s">
         <v>280</v>
       </c>
-      <c r="I39" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J39" s="20" t="s">
+      <c r="I39" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J39" s="19" t="s">
         <v>320</v>
       </c>
-      <c r="K39" s="20" t="s">
+      <c r="K39" s="19" t="s">
         <v>365</v>
       </c>
-      <c r="L39" s="20">
+      <c r="L39" s="19">
         <v>1</v>
       </c>
-      <c r="M39" s="21">
+      <c r="M39" s="20">
         <v>0.38137500000000002</v>
       </c>
-      <c r="N39" s="48">
+      <c r="N39" s="46">
         <f t="shared" si="1"/>
         <v>0.38137500000000002</v>
       </c>
-      <c r="O39" s="20"/>
+      <c r="O39" s="19"/>
     </row>
     <row r="40" spans="1:15" ht="36" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
@@ -3615,7 +3599,7 @@
         <f>ROW(B40) - ROW($B$7)</f>
         <v>33</v>
       </c>
-      <c r="C40" s="22" t="s">
+      <c r="C40" s="21" t="s">
         <v>15</v>
       </c>
       <c r="D40" s="14" t="s">
@@ -3633,7 +3617,7 @@
       <c r="H40" s="14" t="s">
         <v>281</v>
       </c>
-      <c r="I40" s="20" t="s">
+      <c r="I40" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J40" s="14" t="s">
@@ -3648,7 +3632,7 @@
       <c r="M40" s="15">
         <v>6.93E-2</v>
       </c>
-      <c r="N40" s="48">
+      <c r="N40" s="46">
         <f t="shared" si="1"/>
         <v>0.1386</v>
       </c>
@@ -3660,44 +3644,44 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C41" s="23" t="s">
+      <c r="C41" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D41" s="20" t="s">
+      <c r="D41" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="E41" s="20" t="s">
+      <c r="E41" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F41" s="20" t="s">
+      <c r="F41" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="G41" s="20" t="s">
+      <c r="G41" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="H41" s="20" t="s">
+      <c r="H41" s="19" t="s">
         <v>281</v>
       </c>
-      <c r="I41" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J41" s="20" t="s">
+      <c r="I41" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J41" s="19" t="s">
         <v>322</v>
       </c>
       <c r="K41" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L41" s="20">
+      <c r="L41" s="19">
         <v>2</v>
       </c>
-      <c r="M41" s="21">
+      <c r="M41" s="20">
         <v>7.5600000000000001E-2</v>
       </c>
-      <c r="N41" s="48">
+      <c r="N41" s="46">
         <f t="shared" si="1"/>
         <v>0.1512</v>
       </c>
-      <c r="O41" s="20"/>
+      <c r="O41" s="19"/>
     </row>
     <row r="42" spans="1:15" ht="48" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
@@ -3705,7 +3689,7 @@
         <f>ROW(B42) - ROW($B$7)</f>
         <v>35</v>
       </c>
-      <c r="C42" s="22" t="s">
+      <c r="C42" s="21" t="s">
         <v>15</v>
       </c>
       <c r="D42" s="14" t="s">
@@ -3723,7 +3707,7 @@
       <c r="H42" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="I42" s="20" t="s">
+      <c r="I42" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J42" s="14" t="s">
@@ -3738,7 +3722,7 @@
       <c r="M42" s="15">
         <v>0.142875</v>
       </c>
-      <c r="N42" s="48">
+      <c r="N42" s="46">
         <f t="shared" si="1"/>
         <v>0.28575</v>
       </c>
@@ -3750,44 +3734,44 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C43" s="23" t="s">
+      <c r="C43" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="D43" s="20" t="s">
+      <c r="D43" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="E43" s="20" t="s">
+      <c r="E43" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="F43" s="20" t="s">
+      <c r="F43" s="19" t="s">
         <v>395</v>
       </c>
-      <c r="G43" s="20" t="s">
+      <c r="G43" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="H43" s="20" t="s">
+      <c r="H43" s="19" t="s">
         <v>283</v>
       </c>
-      <c r="I43" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J43" s="20" t="s">
+      <c r="I43" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J43" s="19" t="s">
         <v>324</v>
       </c>
       <c r="K43" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L43" s="20">
+      <c r="L43" s="19">
         <v>1</v>
       </c>
-      <c r="M43" s="21">
+      <c r="M43" s="20">
         <v>0.673875</v>
       </c>
-      <c r="N43" s="48">
+      <c r="N43" s="46">
         <f t="shared" si="1"/>
         <v>0.673875</v>
       </c>
-      <c r="O43" s="20"/>
+      <c r="O43" s="19"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
@@ -3795,44 +3779,44 @@
         <f>ROW(B44) - ROW($B$7)</f>
         <v>37</v>
       </c>
-      <c r="C44" s="22" t="s">
+      <c r="C44" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="D44" s="41" t="s">
+      <c r="D44" s="40" t="s">
         <v>66</v>
       </c>
-      <c r="E44" s="41" t="s">
+      <c r="E44" s="40" t="s">
         <v>135</v>
       </c>
-      <c r="F44" s="41" t="s">
+      <c r="F44" s="40" t="s">
         <v>395</v>
       </c>
-      <c r="G44" s="41" t="s">
+      <c r="G44" s="40" t="s">
         <v>191</v>
       </c>
-      <c r="H44" s="41" t="s">
-        <v>389</v>
-      </c>
-      <c r="I44" s="41" t="s">
-        <v>389</v>
-      </c>
-      <c r="J44" s="41" t="s">
-        <v>389</v>
-      </c>
-      <c r="K44" s="41" t="s">
-        <v>389</v>
-      </c>
-      <c r="L44" s="41">
+      <c r="H44" s="40" t="s">
+        <v>389</v>
+      </c>
+      <c r="I44" s="40" t="s">
+        <v>389</v>
+      </c>
+      <c r="J44" s="40" t="s">
+        <v>389</v>
+      </c>
+      <c r="K44" s="40" t="s">
+        <v>389</v>
+      </c>
+      <c r="L44" s="40">
         <v>4</v>
       </c>
-      <c r="M44" s="42">
+      <c r="M44" s="41">
         <v>0</v>
       </c>
-      <c r="N44" s="48">
+      <c r="N44" s="46">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O44" s="43" t="s">
+      <c r="O44" s="42" t="s">
         <v>399</v>
       </c>
     </row>
@@ -3842,44 +3826,44 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C45" s="23" t="s">
+      <c r="C45" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D45" s="20" t="s">
+      <c r="D45" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="E45" s="20" t="s">
+      <c r="E45" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="F45" s="20" t="s">
+      <c r="F45" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="G45" s="20" t="s">
+      <c r="G45" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="H45" s="20" t="s">
+      <c r="H45" s="19" t="s">
         <v>270</v>
       </c>
-      <c r="I45" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J45" s="20" t="s">
+      <c r="I45" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J45" s="19" t="s">
         <v>325</v>
       </c>
       <c r="K45" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L45" s="20">
+      <c r="L45" s="19">
         <v>2</v>
       </c>
-      <c r="M45" s="21">
+      <c r="M45" s="20">
         <v>5.5350000000000003E-2</v>
       </c>
-      <c r="N45" s="48">
+      <c r="N45" s="46">
         <f t="shared" si="1"/>
         <v>0.11070000000000001</v>
       </c>
-      <c r="O45" s="20"/>
+      <c r="O45" s="19"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
@@ -3887,7 +3871,7 @@
         <f>ROW(B46) - ROW($B$7)</f>
         <v>39</v>
       </c>
-      <c r="C46" s="22"/>
+      <c r="C46" s="21"/>
       <c r="D46" s="14" t="s">
         <v>68</v>
       </c>
@@ -3903,7 +3887,7 @@
       <c r="H46" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I46" s="20" t="s">
+      <c r="I46" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J46" s="14" t="s">
@@ -3918,7 +3902,7 @@
       <c r="M46" s="15">
         <v>5.1975E-2</v>
       </c>
-      <c r="N46" s="48">
+      <c r="N46" s="46">
         <f t="shared" si="1"/>
         <v>5.1975E-2</v>
       </c>
@@ -3930,44 +3914,44 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C47" s="23" t="s">
+      <c r="C47" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="D47" s="20" t="s">
+      <c r="D47" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="E47" s="20" t="s">
+      <c r="E47" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="F47" s="20" t="s">
+      <c r="F47" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="G47" s="20" t="s">
+      <c r="G47" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="H47" s="20" t="s">
+      <c r="H47" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="I47" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J47" s="20" t="s">
+      <c r="I47" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J47" s="19" t="s">
         <v>326</v>
       </c>
-      <c r="K47" s="20" t="s">
+      <c r="K47" s="19" t="s">
         <v>367</v>
       </c>
-      <c r="L47" s="20">
+      <c r="L47" s="19">
         <v>1</v>
       </c>
-      <c r="M47" s="21">
+      <c r="M47" s="20">
         <v>2.6999999999999997E-3</v>
       </c>
-      <c r="N47" s="48">
+      <c r="N47" s="46">
         <f t="shared" si="1"/>
         <v>2.6999999999999997E-3</v>
       </c>
-      <c r="O47" s="20"/>
+      <c r="O47" s="19"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
@@ -3975,7 +3959,7 @@
         <f>ROW(B48) - ROW($B$7)</f>
         <v>41</v>
       </c>
-      <c r="C48" s="22" t="s">
+      <c r="C48" s="21" t="s">
         <v>19</v>
       </c>
       <c r="D48" s="14" t="s">
@@ -3993,7 +3977,7 @@
       <c r="H48" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I48" s="20" t="s">
+      <c r="I48" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J48" s="14" t="s">
@@ -4008,7 +3992,7 @@
       <c r="M48" s="15">
         <v>4.6799999999999994E-2</v>
       </c>
-      <c r="N48" s="48">
+      <c r="N48" s="46">
         <f t="shared" si="1"/>
         <v>4.6799999999999994E-2</v>
       </c>
@@ -4020,44 +4004,44 @@
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C49" s="23" t="s">
+      <c r="C49" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="D49" s="20" t="s">
+      <c r="D49" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="E49" s="20" t="s">
+      <c r="E49" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="F49" s="20" t="s">
+      <c r="F49" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="G49" s="20" t="s">
+      <c r="G49" s="19" t="s">
         <v>241</v>
       </c>
-      <c r="H49" s="20" t="s">
+      <c r="H49" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="I49" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J49" s="20" t="s">
+      <c r="I49" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J49" s="19" t="s">
         <v>328</v>
       </c>
-      <c r="K49" s="20" t="s">
+      <c r="K49" s="19" t="s">
         <v>369</v>
       </c>
-      <c r="L49" s="20">
+      <c r="L49" s="19">
         <v>12</v>
       </c>
-      <c r="M49" s="21">
+      <c r="M49" s="20">
         <v>2.2500000000000003E-3</v>
       </c>
-      <c r="N49" s="48">
+      <c r="N49" s="46">
         <f t="shared" si="1"/>
         <v>2.7000000000000003E-2</v>
       </c>
-      <c r="O49" s="20"/>
+      <c r="O49" s="19"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
@@ -4065,7 +4049,7 @@
         <f>ROW(B50) - ROW($B$7)</f>
         <v>43</v>
       </c>
-      <c r="C50" s="22" t="s">
+      <c r="C50" s="21" t="s">
         <v>19</v>
       </c>
       <c r="D50" s="14" t="s">
@@ -4083,7 +4067,7 @@
       <c r="H50" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I50" s="20" t="s">
+      <c r="I50" s="19" t="s">
         <v>389</v>
       </c>
       <c r="J50" s="14" t="s">
@@ -4098,7 +4082,7 @@
       <c r="M50" s="15">
         <v>1.3499999999999999E-3</v>
       </c>
-      <c r="N50" s="48">
+      <c r="N50" s="46">
         <f t="shared" si="1"/>
         <v>2.6999999999999997E-3</v>
       </c>
@@ -4110,42 +4094,42 @@
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="C51" s="23" t="s">
+      <c r="C51" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="D51" s="20" t="s">
+      <c r="D51" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="E51" s="20" t="s">
+      <c r="E51" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="F51" s="20" t="s">
+      <c r="F51" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="G51" s="20" t="s">
+      <c r="G51" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="H51" s="20" t="s">
+      <c r="H51" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="I51" s="20"/>
-      <c r="J51" s="20" t="s">
+      <c r="I51" s="19"/>
+      <c r="J51" s="19" t="s">
         <v>330</v>
       </c>
-      <c r="K51" s="20" t="s">
+      <c r="K51" s="19" t="s">
         <v>371</v>
       </c>
-      <c r="L51" s="20">
+      <c r="L51" s="19">
         <v>8</v>
       </c>
-      <c r="M51" s="21">
+      <c r="M51" s="20">
         <v>2.6999999999999997E-3</v>
       </c>
-      <c r="N51" s="48">
+      <c r="N51" s="46">
         <f t="shared" si="1"/>
         <v>2.1599999999999998E-2</v>
       </c>
-      <c r="O51" s="20"/>
+      <c r="O51" s="19"/>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
@@ -4153,7 +4137,7 @@
         <f>ROW(B52) - ROW($B$7)</f>
         <v>45</v>
       </c>
-      <c r="C52" s="22" t="s">
+      <c r="C52" s="21" t="s">
         <v>19</v>
       </c>
       <c r="D52" s="14" t="s">
@@ -4184,7 +4168,7 @@
       <c r="M52" s="15">
         <v>2.0249999999999999E-3</v>
       </c>
-      <c r="N52" s="48">
+      <c r="N52" s="46">
         <f t="shared" si="1"/>
         <v>4.0499999999999998E-3</v>
       </c>
@@ -4196,42 +4180,42 @@
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="C53" s="22" t="s">
+      <c r="C53" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="D53" s="20" t="s">
+      <c r="D53" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="E53" s="20" t="s">
+      <c r="E53" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="F53" s="20" t="s">
+      <c r="F53" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="G53" s="20" t="s">
+      <c r="G53" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="H53" s="20" t="s">
+      <c r="H53" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="I53" s="20"/>
-      <c r="J53" s="20" t="s">
+      <c r="I53" s="19"/>
+      <c r="J53" s="19" t="s">
         <v>332</v>
       </c>
-      <c r="K53" s="20" t="s">
+      <c r="K53" s="19" t="s">
         <v>373</v>
       </c>
-      <c r="L53" s="20">
+      <c r="L53" s="19">
         <v>4</v>
       </c>
-      <c r="M53" s="21">
+      <c r="M53" s="20">
         <v>2.9249999999999996E-3</v>
       </c>
-      <c r="N53" s="48">
+      <c r="N53" s="46">
         <f t="shared" si="1"/>
         <v>1.1699999999999999E-2</v>
       </c>
-      <c r="O53" s="20"/>
+      <c r="O53" s="19"/>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
@@ -4239,7 +4223,7 @@
         <f>ROW(B54) - ROW($B$7)</f>
         <v>47</v>
       </c>
-      <c r="C54" s="22" t="s">
+      <c r="C54" s="21" t="s">
         <v>19</v>
       </c>
       <c r="D54" s="14" t="s">
@@ -4251,7 +4235,7 @@
       <c r="F54" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="G54" s="41" t="s">
+      <c r="G54" s="40" t="s">
         <v>246</v>
       </c>
       <c r="H54" s="14" t="s">
@@ -4272,7 +4256,7 @@
       <c r="M54" s="15">
         <v>4.5000000000000005E-3</v>
       </c>
-      <c r="N54" s="48">
+      <c r="N54" s="46">
         <f t="shared" si="1"/>
         <v>4.5000000000000005E-3</v>
       </c>
@@ -4284,44 +4268,44 @@
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="C55" s="23" t="s">
+      <c r="C55" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="D55" s="20" t="s">
+      <c r="D55" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="E55" s="20" t="s">
+      <c r="E55" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="F55" s="20" t="s">
+      <c r="F55" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="G55" s="44" t="s">
+      <c r="G55" s="43" t="s">
         <v>247</v>
       </c>
-      <c r="H55" s="20" t="s">
+      <c r="H55" s="19" t="s">
         <v>284</v>
       </c>
-      <c r="I55" s="20" t="s">
+      <c r="I55" s="19" t="s">
         <v>405</v>
       </c>
-      <c r="J55" s="20" t="s">
+      <c r="J55" s="19" t="s">
         <v>404</v>
       </c>
-      <c r="K55" s="20" t="s">
+      <c r="K55" s="19" t="s">
         <v>375</v>
       </c>
-      <c r="L55" s="20">
+      <c r="L55" s="19">
         <v>2</v>
       </c>
-      <c r="M55" s="21">
+      <c r="M55" s="20">
         <v>0.18022500000000002</v>
       </c>
-      <c r="N55" s="48">
+      <c r="N55" s="46">
         <f t="shared" si="1"/>
         <v>0.36045000000000005</v>
       </c>
-      <c r="O55" s="20"/>
+      <c r="O55" s="19"/>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
@@ -4329,7 +4313,7 @@
         <f>ROW(B56) - ROW($B$7)</f>
         <v>49</v>
       </c>
-      <c r="C56" s="23" t="s">
+      <c r="C56" s="22" t="s">
         <v>19</v>
       </c>
       <c r="D56" s="14" t="s">
@@ -4360,7 +4344,7 @@
       <c r="M56" s="15">
         <v>2.6999999999999997E-3</v>
       </c>
-      <c r="N56" s="48">
+      <c r="N56" s="46">
         <f t="shared" si="1"/>
         <v>5.3999999999999994E-3</v>
       </c>
@@ -4372,42 +4356,42 @@
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="C57" s="23" t="s">
+      <c r="C57" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="D57" s="20" t="s">
+      <c r="D57" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="E57" s="20" t="s">
+      <c r="E57" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="F57" s="20" t="s">
+      <c r="F57" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="G57" s="20" t="s">
+      <c r="G57" s="19" t="s">
         <v>249</v>
       </c>
-      <c r="H57" s="20" t="s">
+      <c r="H57" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="I57" s="20"/>
-      <c r="J57" s="20" t="s">
+      <c r="I57" s="19"/>
+      <c r="J57" s="19" t="s">
         <v>334</v>
       </c>
-      <c r="K57" s="20" t="s">
+      <c r="K57" s="19" t="s">
         <v>377</v>
       </c>
-      <c r="L57" s="20">
+      <c r="L57" s="19">
         <v>4</v>
       </c>
-      <c r="M57" s="21">
+      <c r="M57" s="20">
         <v>4.7024999999999997E-2</v>
       </c>
-      <c r="N57" s="48">
+      <c r="N57" s="46">
         <f t="shared" si="1"/>
         <v>0.18809999999999999</v>
       </c>
-      <c r="O57" s="20"/>
+      <c r="O57" s="19"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
@@ -4415,7 +4399,7 @@
         <f>ROW(B58) - ROW($B$7)</f>
         <v>51</v>
       </c>
-      <c r="C58" s="22" t="s">
+      <c r="C58" s="21" t="s">
         <v>19</v>
       </c>
       <c r="D58" s="14" t="s">
@@ -4446,7 +4430,7 @@
       <c r="M58" s="15">
         <v>0.30712500000000004</v>
       </c>
-      <c r="N58" s="48">
+      <c r="N58" s="46">
         <f t="shared" si="1"/>
         <v>0.30712500000000004</v>
       </c>
@@ -4458,44 +4442,44 @@
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="C59" s="23" t="s">
+      <c r="C59" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="D59" s="20" t="s">
+      <c r="D59" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="E59" s="20" t="s">
+      <c r="E59" s="19" t="s">
         <v>150</v>
       </c>
-      <c r="F59" s="20" t="s">
+      <c r="F59" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="G59" s="44" t="s">
+      <c r="G59" s="43" t="s">
         <v>251</v>
       </c>
-      <c r="H59" s="20" t="s">
+      <c r="H59" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="I59" s="20" t="s">
+      <c r="I59" s="19" t="s">
         <v>407</v>
       </c>
-      <c r="J59" s="20" t="s">
+      <c r="J59" s="19" t="s">
         <v>406</v>
       </c>
-      <c r="K59" s="20" t="s">
+      <c r="K59" s="19" t="s">
         <v>379</v>
       </c>
-      <c r="L59" s="20">
+      <c r="L59" s="19">
         <v>3</v>
       </c>
-      <c r="M59" s="21">
+      <c r="M59" s="20">
         <v>2.2500000000000003E-3</v>
       </c>
-      <c r="N59" s="48">
+      <c r="N59" s="46">
         <f t="shared" si="1"/>
         <v>6.7500000000000008E-3</v>
       </c>
-      <c r="O59" s="20"/>
+      <c r="O59" s="19"/>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
@@ -4503,7 +4487,7 @@
         <f>ROW(B60) - ROW($B$7)</f>
         <v>53</v>
       </c>
-      <c r="C60" s="22" t="s">
+      <c r="C60" s="21" t="s">
         <v>19</v>
       </c>
       <c r="D60" s="14" t="s">
@@ -4536,7 +4520,7 @@
       <c r="M60" s="15">
         <v>2.6999999999999997E-3</v>
       </c>
-      <c r="N60" s="48">
+      <c r="N60" s="46">
         <f t="shared" si="1"/>
         <v>5.3999999999999994E-3</v>
       </c>
@@ -4548,42 +4532,42 @@
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="C61" s="23" t="s">
+      <c r="C61" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="D61" s="20" t="s">
+      <c r="D61" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="E61" s="20" t="s">
+      <c r="E61" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="F61" s="20" t="s">
+      <c r="F61" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="G61" s="20" t="s">
+      <c r="G61" s="19" t="s">
         <v>253</v>
       </c>
-      <c r="H61" s="20" t="s">
+      <c r="H61" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="I61" s="20"/>
-      <c r="J61" s="20" t="s">
+      <c r="I61" s="19"/>
+      <c r="J61" s="19" t="s">
         <v>337</v>
       </c>
-      <c r="K61" s="20" t="s">
+      <c r="K61" s="19" t="s">
         <v>381</v>
       </c>
-      <c r="L61" s="20">
+      <c r="L61" s="19">
         <v>1</v>
       </c>
-      <c r="M61" s="21">
+      <c r="M61" s="20">
         <v>2.6999999999999997E-3</v>
       </c>
-      <c r="N61" s="48">
+      <c r="N61" s="46">
         <f t="shared" si="1"/>
         <v>2.6999999999999997E-3</v>
       </c>
-      <c r="O61" s="20"/>
+      <c r="O61" s="19"/>
     </row>
     <row r="62" spans="1:15" ht="48" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
@@ -4591,7 +4575,7 @@
         <f>ROW(B62) - ROW($B$7)</f>
         <v>55</v>
       </c>
-      <c r="C62" s="22" t="s">
+      <c r="C62" s="21" t="s">
         <v>21</v>
       </c>
       <c r="D62" s="14" t="s">
@@ -4622,7 +4606,7 @@
       <c r="M62" s="15">
         <v>4.4324999999999996E-2</v>
       </c>
-      <c r="N62" s="48">
+      <c r="N62" s="46">
         <f t="shared" si="1"/>
         <v>8.8649999999999993E-2</v>
       </c>
@@ -4634,44 +4618,44 @@
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="C63" s="23" t="s">
+      <c r="C63" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="D63" s="20" t="s">
+      <c r="D63" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="E63" s="20" t="s">
+      <c r="E63" s="19" t="s">
         <v>154</v>
       </c>
       <c r="F63" s="14" t="s">
         <v>395</v>
       </c>
-      <c r="G63" s="20" t="s">
+      <c r="G63" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="H63" s="20" t="s">
+      <c r="H63" s="19" t="s">
         <v>286</v>
       </c>
-      <c r="I63" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="J63" s="20" t="s">
+      <c r="I63" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="J63" s="19" t="s">
         <v>389</v>
       </c>
       <c r="K63" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L63" s="20">
+      <c r="L63" s="19">
         <v>1</v>
       </c>
-      <c r="M63" s="21">
+      <c r="M63" s="20">
         <v>81.627750000000006</v>
       </c>
-      <c r="N63" s="48">
+      <c r="N63" s="46">
         <f t="shared" si="1"/>
         <v>81.627750000000006</v>
       </c>
-      <c r="O63" s="20"/>
+      <c r="O63" s="19"/>
     </row>
     <row r="64" spans="1:15" ht="48" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
@@ -4679,7 +4663,7 @@
         <f>ROW(B64) - ROW($B$7)</f>
         <v>57</v>
       </c>
-      <c r="C64" s="22" t="s">
+      <c r="C64" s="21" t="s">
         <v>23</v>
       </c>
       <c r="D64" s="14" t="s">
@@ -4710,7 +4694,7 @@
       <c r="M64" s="15">
         <v>0.59602500000000003</v>
       </c>
-      <c r="N64" s="48">
+      <c r="N64" s="46">
         <f t="shared" si="1"/>
         <v>0.59602500000000003</v>
       </c>
@@ -4722,42 +4706,42 @@
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="C65" s="23" t="s">
+      <c r="C65" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D65" s="20" t="s">
+      <c r="D65" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="E65" s="20" t="s">
+      <c r="E65" s="19" t="s">
         <v>156</v>
       </c>
       <c r="F65" s="14" t="s">
         <v>395</v>
       </c>
-      <c r="G65" s="20" t="s">
+      <c r="G65" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="H65" s="20" t="s">
+      <c r="H65" s="19" t="s">
         <v>287</v>
       </c>
-      <c r="I65" s="20"/>
-      <c r="J65" s="20" t="s">
+      <c r="I65" s="19"/>
+      <c r="J65" s="19" t="s">
         <v>340</v>
       </c>
       <c r="K65" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L65" s="20">
+      <c r="L65" s="19">
         <v>1</v>
       </c>
-      <c r="M65" s="21">
+      <c r="M65" s="20">
         <v>0.172125</v>
       </c>
-      <c r="N65" s="48">
+      <c r="N65" s="46">
         <f t="shared" si="1"/>
         <v>0.172125</v>
       </c>
-      <c r="O65" s="20"/>
+      <c r="O65" s="19"/>
     </row>
     <row r="66" spans="1:15" ht="36" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
@@ -4765,7 +4749,7 @@
         <f>ROW(B66) - ROW($B$7)</f>
         <v>59</v>
       </c>
-      <c r="C66" s="22" t="s">
+      <c r="C66" s="21" t="s">
         <v>24</v>
       </c>
       <c r="D66" s="14" t="s">
@@ -4796,7 +4780,7 @@
       <c r="M66" s="15">
         <v>9.3375E-2</v>
       </c>
-      <c r="N66" s="48">
+      <c r="N66" s="46">
         <f t="shared" si="1"/>
         <v>9.3375E-2</v>
       </c>
@@ -4808,42 +4792,42 @@
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="C67" s="23" t="s">
+      <c r="C67" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D67" s="20" t="s">
+      <c r="D67" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="E67" s="20" t="s">
+      <c r="E67" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="F67" s="20" t="s">
+      <c r="F67" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="G67" s="20" t="s">
+      <c r="G67" s="19" t="s">
         <v>255</v>
       </c>
-      <c r="H67" s="20" t="s">
+      <c r="H67" s="19" t="s">
         <v>288</v>
       </c>
-      <c r="I67" s="20"/>
-      <c r="J67" s="20" t="s">
+      <c r="I67" s="19"/>
+      <c r="J67" s="19" t="s">
         <v>342</v>
       </c>
       <c r="K67" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L67" s="20">
+      <c r="L67" s="19">
         <v>1</v>
       </c>
-      <c r="M67" s="21">
+      <c r="M67" s="20">
         <v>1.111275</v>
       </c>
-      <c r="N67" s="48">
+      <c r="N67" s="46">
         <f t="shared" si="1"/>
         <v>1.111275</v>
       </c>
-      <c r="O67" s="20"/>
+      <c r="O67" s="19"/>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
@@ -4851,7 +4835,7 @@
         <f>ROW(B68) - ROW($B$7)</f>
         <v>61</v>
       </c>
-      <c r="C68" s="22" t="s">
+      <c r="C68" s="21" t="s">
         <v>25</v>
       </c>
       <c r="D68" s="14" t="s">
@@ -4882,7 +4866,7 @@
       <c r="M68" s="15">
         <v>0.38632499999999997</v>
       </c>
-      <c r="N68" s="48">
+      <c r="N68" s="46">
         <f t="shared" si="1"/>
         <v>0.38632499999999997</v>
       </c>
@@ -4894,42 +4878,42 @@
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="C69" s="23" t="s">
+      <c r="C69" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="D69" s="20" t="s">
+      <c r="D69" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="E69" s="20" t="s">
+      <c r="E69" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="F69" s="20" t="s">
+      <c r="F69" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="G69" s="20" t="s">
+      <c r="G69" s="19" t="s">
         <v>257</v>
       </c>
-      <c r="H69" s="20" t="s">
+      <c r="H69" s="19" t="s">
         <v>290</v>
       </c>
-      <c r="I69" s="20"/>
-      <c r="J69" s="20" t="s">
+      <c r="I69" s="19"/>
+      <c r="J69" s="19" t="s">
         <v>344</v>
       </c>
       <c r="K69" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L69" s="20">
+      <c r="L69" s="19">
         <v>1</v>
       </c>
-      <c r="M69" s="21">
+      <c r="M69" s="20">
         <v>9.7967250000000003</v>
       </c>
-      <c r="N69" s="48">
+      <c r="N69" s="46">
         <f t="shared" si="1"/>
         <v>9.7967250000000003</v>
       </c>
-      <c r="O69" s="20"/>
+      <c r="O69" s="19"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
@@ -4937,7 +4921,7 @@
         <f>ROW(B70) - ROW($B$7)</f>
         <v>63</v>
       </c>
-      <c r="C70" s="22" t="s">
+      <c r="C70" s="21" t="s">
         <v>25</v>
       </c>
       <c r="D70" s="14" t="s">
@@ -4968,7 +4952,7 @@
       <c r="M70" s="15">
         <v>9.018675</v>
       </c>
-      <c r="N70" s="48">
+      <c r="N70" s="46">
         <f t="shared" si="1"/>
         <v>9.018675</v>
       </c>
@@ -4980,42 +4964,42 @@
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
-      <c r="C71" s="23" t="s">
+      <c r="C71" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="D71" s="20" t="s">
+      <c r="D71" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="E71" s="20" t="s">
+      <c r="E71" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="F71" s="20" t="s">
+      <c r="F71" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="G71" s="20" t="s">
+      <c r="G71" s="19" t="s">
         <v>259</v>
       </c>
-      <c r="H71" s="20" t="s">
+      <c r="H71" s="19" t="s">
         <v>292</v>
       </c>
-      <c r="I71" s="20"/>
-      <c r="J71" s="20" t="s">
+      <c r="I71" s="19"/>
+      <c r="J71" s="19" t="s">
         <v>346</v>
       </c>
       <c r="K71" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L71" s="20">
+      <c r="L71" s="19">
         <v>4</v>
       </c>
-      <c r="M71" s="21">
+      <c r="M71" s="20">
         <v>1.8424125</v>
       </c>
-      <c r="N71" s="48">
+      <c r="N71" s="46">
         <f t="shared" si="1"/>
         <v>7.36965</v>
       </c>
-      <c r="O71" s="20"/>
+      <c r="O71" s="19"/>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
@@ -5023,7 +5007,7 @@
         <f>ROW(B72) - ROW($B$7)</f>
         <v>65</v>
       </c>
-      <c r="C72" s="22" t="s">
+      <c r="C72" s="21" t="s">
         <v>25</v>
       </c>
       <c r="D72" s="14" t="s">
@@ -5054,7 +5038,7 @@
       <c r="M72" s="15">
         <v>0.48060000000000003</v>
       </c>
-      <c r="N72" s="48">
+      <c r="N72" s="46">
         <f t="shared" si="1"/>
         <v>0.48060000000000003</v>
       </c>
@@ -5066,42 +5050,42 @@
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
-      <c r="C73" s="23" t="s">
+      <c r="C73" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D73" s="20" t="s">
+      <c r="D73" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="E73" s="20" t="s">
+      <c r="E73" s="19" t="s">
         <v>164</v>
       </c>
-      <c r="F73" s="20" t="s">
+      <c r="F73" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="G73" s="20" t="s">
+      <c r="G73" s="19" t="s">
         <v>261</v>
       </c>
-      <c r="H73" s="20" t="s">
+      <c r="H73" s="19" t="s">
         <v>288</v>
       </c>
-      <c r="I73" s="20"/>
-      <c r="J73" s="20" t="s">
+      <c r="I73" s="19"/>
+      <c r="J73" s="19" t="s">
         <v>348</v>
       </c>
       <c r="K73" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L73" s="20">
+      <c r="L73" s="19">
         <v>1</v>
       </c>
-      <c r="M73" s="21">
+      <c r="M73" s="20">
         <v>1.1843999999999999</v>
       </c>
-      <c r="N73" s="48">
+      <c r="N73" s="46">
         <f t="shared" ref="N73:N77" si="2">M73*L73</f>
         <v>1.1843999999999999</v>
       </c>
-      <c r="O73" s="20"/>
+      <c r="O73" s="19"/>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
@@ -5109,7 +5093,7 @@
         <f>ROW(B74) - ROW($B$7)</f>
         <v>67</v>
       </c>
-      <c r="C74" s="22" t="s">
+      <c r="C74" s="21" t="s">
         <v>28</v>
       </c>
       <c r="D74" s="14" t="s">
@@ -5140,7 +5124,7 @@
       <c r="M74" s="15">
         <v>0.67342500000000005</v>
       </c>
-      <c r="N74" s="48">
+      <c r="N74" s="46">
         <f t="shared" si="2"/>
         <v>0.67342500000000005</v>
       </c>
@@ -5152,42 +5136,42 @@
         <f t="shared" si="0"/>
         <v>68</v>
       </c>
-      <c r="C75" s="23" t="s">
+      <c r="C75" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D75" s="20" t="s">
+      <c r="D75" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="E75" s="20" t="s">
+      <c r="E75" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="F75" s="20" t="s">
+      <c r="F75" s="19" t="s">
         <v>408</v>
       </c>
-      <c r="G75" s="20" t="s">
+      <c r="G75" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="H75" s="20" t="s">
+      <c r="H75" s="19" t="s">
         <v>288</v>
       </c>
-      <c r="I75" s="20"/>
-      <c r="J75" s="20" t="s">
+      <c r="I75" s="19"/>
+      <c r="J75" s="19" t="s">
         <v>387</v>
       </c>
       <c r="K75" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L75" s="20">
+      <c r="L75" s="19">
         <v>2</v>
       </c>
-      <c r="M75" s="21">
+      <c r="M75" s="20">
         <v>0.74317499999999992</v>
       </c>
-      <c r="N75" s="48">
+      <c r="N75" s="46">
         <f t="shared" si="2"/>
         <v>1.4863499999999998</v>
       </c>
-      <c r="O75" s="20"/>
+      <c r="O75" s="19"/>
     </row>
     <row r="76" spans="1:15" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
@@ -5195,42 +5179,42 @@
         <f t="shared" si="0"/>
         <v>69</v>
       </c>
-      <c r="C76" s="23" t="s">
+      <c r="C76" s="22" t="s">
         <v>409</v>
       </c>
-      <c r="D76" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="E76" s="20" t="s">
+      <c r="D76" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="E76" s="19" t="s">
         <v>412</v>
       </c>
-      <c r="F76" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="G76" s="20" t="s">
+      <c r="F76" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="G76" s="19" t="s">
         <v>413</v>
       </c>
-      <c r="H76" s="20" t="s">
+      <c r="H76" s="19" t="s">
         <v>414</v>
       </c>
-      <c r="I76" s="20"/>
-      <c r="J76" s="20" t="s">
+      <c r="I76" s="19"/>
+      <c r="J76" s="19" t="s">
         <v>389</v>
       </c>
       <c r="K76" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L76" s="20">
+      <c r="L76" s="19">
         <v>1</v>
       </c>
-      <c r="M76" s="21">
+      <c r="M76" s="20">
         <v>127.46</v>
       </c>
-      <c r="N76" s="48">
+      <c r="N76" s="46">
         <f t="shared" si="2"/>
         <v>127.46</v>
       </c>
-      <c r="O76" s="46" t="s">
+      <c r="O76" s="45" t="s">
         <v>415</v>
       </c>
     </row>
@@ -5240,40 +5224,40 @@
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="C77" s="23" t="s">
+      <c r="C77" s="22" t="s">
         <v>409</v>
       </c>
-      <c r="D77" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="E77" s="20" t="s">
+      <c r="D77" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="E77" s="19" t="s">
         <v>410</v>
       </c>
-      <c r="F77" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="G77" s="20" t="s">
+      <c r="F77" s="19" t="s">
+        <v>389</v>
+      </c>
+      <c r="G77" s="19" t="s">
         <v>411</v>
       </c>
-      <c r="H77" s="20"/>
-      <c r="I77" s="20"/>
-      <c r="J77" s="20" t="s">
+      <c r="H77" s="19"/>
+      <c r="I77" s="19"/>
+      <c r="J77" s="19" t="s">
         <v>389</v>
       </c>
       <c r="K77" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L77" s="20">
+      <c r="L77" s="19">
         <v>1</v>
       </c>
-      <c r="M77" s="21">
+      <c r="M77" s="20">
         <v>7.01</v>
       </c>
-      <c r="N77" s="48">
+      <c r="N77" s="46">
         <f t="shared" si="2"/>
         <v>7.01</v>
       </c>
-      <c r="O77" s="20"/>
+      <c r="O77" s="19"/>
     </row>
     <row r="78" spans="1:15" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
@@ -5288,32 +5272,17 @@
       <c r="J78" s="1"/>
       <c r="K78" s="1"/>
       <c r="L78" s="1"/>
-      <c r="M78" s="45"/>
+      <c r="M78" s="44"/>
       <c r="N78" s="18">
         <f>SUM(N8:N77)</f>
         <v>259.62174999999996</v>
       </c>
       <c r="O78" s="1"/>
     </row>
-    <row r="79" spans="1:15" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="1"/>
-      <c r="B79" s="1"/>
-      <c r="C79" s="1"/>
-      <c r="D79" s="1"/>
-      <c r="E79" s="1"/>
-      <c r="F79" s="1"/>
-      <c r="G79" s="1"/>
-      <c r="H79" s="1"/>
-      <c r="I79" s="1"/>
-      <c r="J79" s="1"/>
-      <c r="K79" s="1"/>
-      <c r="L79" s="1"/>
-      <c r="M79" s="45"/>
-      <c r="N79" s="19">
-        <f>N78/10</f>
-        <v>25.962174999999995</v>
-      </c>
-      <c r="O79" s="1"/>
+    <row r="99" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D99" s="10"/>
+      <c r="E99" s="10"/>
+      <c r="F99" s="10"/>
     </row>
     <row r="100" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D100" s="10"/>
@@ -5664,11 +5633,6 @@
       <c r="D169" s="10"/>
       <c r="E169" s="10"/>
       <c r="F169" s="10"/>
-    </row>
-    <row r="170" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D170" s="10"/>
-      <c r="E170" s="10"/>
-      <c r="F170" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>